<commit_message>
add new data and wrangle for inclusion into package
</commit_message>
<xml_diff>
--- a/data_prep/1999 Bureau - Apparent digestibility of rendered animal protein ingredients for rainbow trout.xlsx
+++ b/data_prep/1999 Bureau - Apparent digestibility of rendered animal protein ingredients for rainbow trout.xlsx
@@ -5,22 +5,22 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atellbuscher\Documents\R\aquacultuR\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\atellbuscher\Documents\R\aquacultuR\data_prep\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2BB1BE8-C3B0-4905-B581-9282F3B54FB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A81A040-DDC6-468E-B72A-1BF2D75EFA83}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-19320" yWindow="6075" windowWidth="19440" windowHeight="10320" activeTab="4" xr2:uid="{413B3DB9-2031-4BEC-8653-712DE25A4A6C}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{413B3DB9-2031-4BEC-8653-712DE25A4A6C}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet5" sheetId="5" r:id="rId1"/>
+    <sheet name="table 3" sheetId="5" r:id="rId1"/>
     <sheet name="table 4" sheetId="1" r:id="rId2"/>
     <sheet name="table 5" sheetId="2" r:id="rId3"/>
     <sheet name="table 6" sheetId="3" r:id="rId4"/>
     <sheet name="table 7" sheetId="4" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="bTBLFN2" localSheetId="0">Sheet5!$A$6</definedName>
+    <definedName name="bTBLFN2" localSheetId="0">'table 3'!$A$6</definedName>
     <definedName name="bTBLFN3" localSheetId="1">'table 4'!#REF!</definedName>
     <definedName name="bTBLFN4" localSheetId="2">'table 5'!#REF!</definedName>
     <definedName name="bTBLFN5" localSheetId="3">'table 6'!#REF!</definedName>
@@ -217,26 +217,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="47">
   <si>
     <t>Ingredients</t>
   </si>
   <si>
-    <t>DM %</t>
-  </si>
-  <si>
-    <t>CP %</t>
-  </si>
-  <si>
-    <t>Lipid %</t>
-  </si>
-  <si>
-    <t>Ash %</t>
-  </si>
-  <si>
-    <t>GE kJ/g</t>
-  </si>
-  <si>
     <t>Reference A</t>
   </si>
   <si>
@@ -261,18 +246,6 @@
     <t>Reference diet C</t>
   </si>
   <si>
-    <t>ADC DM %</t>
-  </si>
-  <si>
-    <t>ADC CP %</t>
-  </si>
-  <si>
-    <t>ADC GE %</t>
-  </si>
-  <si>
-    <t>ADC Lipid %</t>
-  </si>
-  <si>
     <t>Feather meal 1</t>
   </si>
   <si>
@@ -348,26 +321,50 @@
     <t>Brewer's dried yeast</t>
   </si>
   <si>
-    <t>Vitamin premixa</t>
-  </si>
-  <si>
-    <t>Mineral premixa</t>
-  </si>
-  <si>
     <t>Celite AW 521</t>
   </si>
   <si>
     <t>Fish oil, herring</t>
   </si>
   <si>
-    <t>Total</t>
+    <t>ADC DM</t>
+  </si>
+  <si>
+    <t>ADC CP</t>
+  </si>
+  <si>
+    <t>ADC Lipid</t>
+  </si>
+  <si>
+    <t>ADC GE</t>
+  </si>
+  <si>
+    <t>DM</t>
+  </si>
+  <si>
+    <t>CP</t>
+  </si>
+  <si>
+    <t>Lipid</t>
+  </si>
+  <si>
+    <t>Ash</t>
+  </si>
+  <si>
+    <t>GE_kJ_g</t>
+  </si>
+  <si>
+    <t>Mineral premix</t>
+  </si>
+  <si>
+    <t>Vitamin premix</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -379,14 +376,6 @@
       <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <u/>
-      <sz val="11"/>
-      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -422,9 +411,8 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -434,12 +422,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="2">
-    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -773,133 +758,125 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0D5F7AE7-1FB8-4743-BBDD-E9F6E9E61216}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.7109375" customWidth="1"/>
-    <col min="2" max="2" width="12.42578125" customWidth="1"/>
+    <col min="1" max="1" width="24.6640625" customWidth="1"/>
+    <col min="2" max="2" width="12.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" ht="105" x14ac:dyDescent="0.25">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B2" s="2">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="B3" s="2">
         <v>49</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="B4" s="2">
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="45" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="B5" s="2">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B6" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B7" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="B8" s="2">
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:2" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="B9" s="2">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="B10" s="2">
-        <v>100</v>
-      </c>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A10" s="2"/>
+      <c r="B10" s="2"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="A6" r:id="rId1" location="TBLFN2" display="https://www.sciencedirect.com/science/article/pii/S0044848699002100 - TBLFN2" xr:uid="{E4E26E51-BE87-4504-9636-458EF1AC9675}"/>
-    <hyperlink ref="A7" r:id="rId2" location="TBLFN2" display="https://www.sciencedirect.com/science/article/pii/S0044848699002100 - TBLFN2" xr:uid="{78B6E024-E939-404D-9F1F-A8C20D1C0416}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BDF43D8-CA44-4180-AF58-F39C009C307B}">
   <dimension ref="A1:F24"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="6" width="18.7109375" customWidth="1"/>
+    <col min="1" max="6" width="18.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" ht="30" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
-        <v>6</v>
       </c>
       <c r="B2" s="2">
         <v>95</v>
@@ -917,9 +894,9 @@
         <v>24.6</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="B3" s="2">
         <v>95.9</v>
@@ -937,9 +914,9 @@
         <v>24.1</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="B4" s="2">
         <v>93.9</v>
@@ -948,7 +925,7 @@
         <v>50.4</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E4" s="2">
         <v>7</v>
@@ -957,9 +934,9 @@
         <v>23.9</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B5" s="2">
         <v>90.3</v>
@@ -977,9 +954,9 @@
         <v>25.7</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B6" s="2">
         <v>93.2</v>
@@ -997,9 +974,9 @@
         <v>24.6</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="B7" s="2">
         <v>87.2</v>
@@ -1017,9 +994,9 @@
         <v>26.2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="B8" s="2">
         <v>91.4</v>
@@ -1037,9 +1014,9 @@
         <v>25.8</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="B9" s="2">
         <v>96.3</v>
@@ -1057,9 +1034,9 @@
         <v>19.5</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B10" s="2">
         <v>95.3</v>
@@ -1077,9 +1054,9 @@
         <v>23.3</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="B11" s="2">
         <v>95.9</v>
@@ -1097,9 +1074,9 @@
         <v>20.7</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="B12" s="2">
         <v>95</v>
@@ -1117,9 +1094,9 @@
         <v>17.399999999999999</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="B13" s="2">
         <v>93.1</v>
@@ -1137,9 +1114,9 @@
         <v>18.899999999999999</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B14" s="2">
         <v>96.8</v>
@@ -1157,9 +1134,9 @@
         <v>19.600000000000001</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B15" s="2">
         <v>94</v>
@@ -1177,9 +1154,9 @@
         <v>21.8</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="30" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:6" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B16" s="2">
         <v>97.2</v>
@@ -1197,9 +1174,9 @@
         <v>21.5</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B17" s="2">
         <v>94.4</v>
@@ -1217,9 +1194,9 @@
         <v>25.3</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="B18" s="2">
         <v>89.5</v>
@@ -1237,9 +1214,9 @@
         <v>25.5</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="B19" s="2">
         <v>91.3</v>
@@ -1248,7 +1225,7 @@
         <v>91.4</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E19" s="2">
         <v>5.7</v>
@@ -1257,9 +1234,9 @@
         <v>23.6</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="B20" s="2">
         <v>92.5</v>
@@ -1268,7 +1245,7 @@
         <v>93.2</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E20" s="2">
         <v>4.5999999999999996</v>
@@ -1277,9 +1254,9 @@
         <v>23.9</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B21" s="2">
         <v>92.2</v>
@@ -1288,7 +1265,7 @@
         <v>77.5</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E21" s="2">
         <v>11</v>
@@ -1297,9 +1274,9 @@
         <v>21.7</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B22" s="2">
         <v>96.5</v>
@@ -1308,7 +1285,7 @@
         <v>93.8</v>
       </c>
       <c r="D22" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E22" s="2">
         <v>1.7</v>
@@ -1317,9 +1294,9 @@
         <v>24.7</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B23" s="2">
         <v>93.1</v>
@@ -1328,7 +1305,7 @@
         <v>88.4</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E23" s="2">
         <v>6.9</v>
@@ -1337,9 +1314,9 @@
         <v>23</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B24" s="2">
         <v>91.5</v>
@@ -1348,7 +1325,7 @@
         <v>94</v>
       </c>
       <c r="D24" s="2" t="s">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E24" s="2">
         <v>2.2999999999999998</v>
@@ -1366,35 +1343,35 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3D1D9751-81FA-4899-88B0-6413B6CD4C66}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="24.85546875" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" customWidth="1"/>
-    <col min="3" max="3" width="10.42578125" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" customWidth="1"/>
-    <col min="5" max="5" width="10.85546875" customWidth="1"/>
+    <col min="1" max="1" width="24.88671875" customWidth="1"/>
+    <col min="2" max="2" width="11.109375" customWidth="1"/>
+    <col min="3" max="3" width="10.44140625" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" customWidth="1"/>
+    <col min="5" max="5" width="10.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="B2" s="2">
         <v>83</v>
@@ -1409,9 +1386,9 @@
         <v>86</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B3" s="2">
         <v>82</v>
@@ -1426,9 +1403,9 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="B4" s="2">
         <v>80</v>
@@ -1443,9 +1420,9 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="B5" s="2">
         <v>79</v>
@@ -1460,9 +1437,9 @@
         <v>76</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>21</v>
+        <v>12</v>
       </c>
       <c r="B6" s="2">
         <v>84</v>
@@ -1477,9 +1454,9 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="B7" s="2">
         <v>61</v>
@@ -1494,9 +1471,9 @@
         <v>68</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="B8" s="2">
         <v>72</v>
@@ -1511,9 +1488,9 @@
         <v>73</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="B9" s="2">
         <v>76</v>
@@ -1537,35 +1514,35 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CCEA7521-BD2C-49FF-9E83-A914395B8B1E}">
   <dimension ref="A1:E9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="26.7109375" customWidth="1"/>
-    <col min="2" max="2" width="11.140625" customWidth="1"/>
-    <col min="3" max="3" width="11.5703125" customWidth="1"/>
-    <col min="4" max="4" width="12.140625" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
+    <col min="1" max="1" width="26.6640625" customWidth="1"/>
+    <col min="2" max="2" width="11.109375" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" customWidth="1"/>
+    <col min="4" max="4" width="12.109375" customWidth="1"/>
+    <col min="5" max="5" width="12.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>17</v>
+        <v>38</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="B2" s="2">
         <v>84</v>
@@ -1580,9 +1557,9 @@
         <v>88</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="B3" s="2">
         <v>72</v>
@@ -1597,9 +1574,9 @@
         <v>82</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="B4" s="2">
         <v>66</v>
@@ -1614,9 +1591,9 @@
         <v>76</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="B5" s="2">
         <v>70</v>
@@ -1631,9 +1608,9 @@
         <v>82</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>27</v>
+        <v>18</v>
       </c>
       <c r="B6" s="2">
         <v>70</v>
@@ -1648,9 +1625,9 @@
         <v>83</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="B7" s="2">
         <v>77</v>
@@ -1665,9 +1642,9 @@
         <v>87</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="B8" s="2">
         <v>82</v>
@@ -1682,9 +1659,9 @@
         <v>82</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="B9" s="2">
         <v>87</v>
@@ -1708,31 +1685,31 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3888B016-3805-4C42-980A-2D3181E69717}">
   <dimension ref="A1:D8"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.5703125" customWidth="1"/>
-    <col min="2" max="2" width="11.28515625" customWidth="1"/>
+    <col min="1" max="1" width="15.5546875" customWidth="1"/>
+    <col min="2" max="2" width="11.33203125" customWidth="1"/>
     <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>14</v>
+        <v>36</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>15</v>
+        <v>37</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="B2" s="2">
         <v>87</v>
@@ -1744,9 +1721,9 @@
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>32</v>
+        <v>23</v>
       </c>
       <c r="B3" s="2">
         <v>92</v>
@@ -1758,9 +1735,9 @@
         <v>92</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>33</v>
+        <v>24</v>
       </c>
       <c r="B4" s="2">
         <v>92</v>
@@ -1772,9 +1749,9 @@
         <v>93</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="B5" s="2">
         <v>99</v>
@@ -1786,9 +1763,9 @@
         <v>99</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>35</v>
+        <v>26</v>
       </c>
       <c r="B6" s="2">
         <v>79</v>
@@ -1800,9 +1777,9 @@
         <v>79</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>36</v>
+        <v>27</v>
       </c>
       <c r="B7" s="2">
         <v>94</v>
@@ -1814,9 +1791,9 @@
         <v>94</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="B8" s="2">
         <v>87</v>

</xml_diff>